<commit_message>
Update README with the phase model, new screens and a 15-minute demo script; refresh demo workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ioDNqWqmysS8ePdYhJWTc
</commit_message>
<xml_diff>
--- a/demo-assets/InvestmentsToolMapping_SYNTHETIC.xlsx
+++ b/demo-assets/InvestmentsToolMapping_SYNTHETIC.xlsx
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -484,10 +484,10 @@
         <v>Ops</v>
       </c>
       <c r="G2" t="str">
-        <v>Other</v>
+        <v>Risk</v>
       </c>
       <c r="H2" t="str">
-        <v>NON-Inv</v>
+        <v>Risk Analytics</v>
       </c>
       <c r="I2">
         <v>420</v>
@@ -542,10 +542,10 @@
         <v>Ops</v>
       </c>
       <c r="G4" t="str">
-        <v>Other</v>
+        <v>PM</v>
       </c>
       <c r="H4" t="str">
-        <v>NON-Inv</v>
+        <v>Cash Management</v>
       </c>
       <c r="I4">
         <v>95</v>
@@ -574,7 +574,7 @@
         <v>Other</v>
       </c>
       <c r="H5" t="str">
-        <v>NON-Inv</v>
+        <v>Integration</v>
       </c>
       <c r="I5">
         <v>60</v>
@@ -603,7 +603,7 @@
         <v>Other</v>
       </c>
       <c r="H6" t="str">
-        <v>NON-Inv</v>
+        <v>Integration</v>
       </c>
       <c r="I6">
         <v>45</v>
@@ -632,7 +632,7 @@
         <v>PM</v>
       </c>
       <c r="H7" t="str">
-        <v>Portfolio Management</v>
+        <v>Order Management</v>
       </c>
       <c r="I7">
         <v>1250</v>
@@ -661,7 +661,7 @@
         <v>PM</v>
       </c>
       <c r="H8" t="str">
-        <v>Portfolio Management</v>
+        <v>Order Management</v>
       </c>
       <c r="I8">
         <v>900</v>
@@ -690,7 +690,7 @@
         <v>PM</v>
       </c>
       <c r="H9" t="str">
-        <v>Portfolio Management</v>
+        <v>Order Management</v>
       </c>
       <c r="I9">
         <v>1400</v>
@@ -745,10 +745,10 @@
         <v>Inv</v>
       </c>
       <c r="G11" t="str">
-        <v>PM</v>
+        <v>Trading</v>
       </c>
       <c r="H11" t="str">
-        <v>Portfolio Management</v>
+        <v>Execution</v>
       </c>
       <c r="I11">
         <v>380</v>
@@ -777,7 +777,7 @@
         <v>PM</v>
       </c>
       <c r="H12" t="str">
-        <v>Portfolio Management</v>
+        <v>Portfolio Construction</v>
       </c>
       <c r="I12">
         <v>260</v>
@@ -806,7 +806,7 @@
         <v>Trading</v>
       </c>
       <c r="H13" t="str">
-        <v>Execution</v>
+        <v>Market Data</v>
       </c>
       <c r="I13">
         <v>2100</v>
@@ -835,7 +835,7 @@
         <v>PM</v>
       </c>
       <c r="H14" t="str">
-        <v>Portfolio Management</v>
+        <v>Order Management</v>
       </c>
       <c r="I14">
         <v>640</v>
@@ -864,7 +864,7 @@
         <v>PM</v>
       </c>
       <c r="H15" t="str">
-        <v>Manage Portfolio</v>
+        <v>Portfolio Construction</v>
       </c>
       <c r="I15">
         <v>310</v>
@@ -890,10 +890,10 @@
         <v>Inv</v>
       </c>
       <c r="G16" t="str">
-        <v>Other</v>
+        <v>PM</v>
       </c>
       <c r="H16" t="str">
-        <v>Tech</v>
+        <v>Optimisation</v>
       </c>
       <c r="I16">
         <v>150</v>
@@ -919,10 +919,10 @@
         <v>Inv</v>
       </c>
       <c r="G17" t="str">
-        <v>Other</v>
+        <v>Trading</v>
       </c>
       <c r="H17" t="str">
-        <v>NON-Inv</v>
+        <v>Market Data</v>
       </c>
       <c r="I17">
         <v>85</v>
@@ -951,7 +951,7 @@
         <v>Other</v>
       </c>
       <c r="H18" t="str">
-        <v>NON-Inv</v>
+        <v>Integration</v>
       </c>
       <c r="I18">
         <v>70</v>
@@ -980,7 +980,7 @@
         <v>Other</v>
       </c>
       <c r="H19" t="str">
-        <v>NON-Inv</v>
+        <v>Data Platform</v>
       </c>
       <c r="I19">
         <v>55</v>
@@ -1009,7 +1009,7 @@
         <v>Other</v>
       </c>
       <c r="H20" t="str">
-        <v>NON-Inv</v>
+        <v>Data Platform</v>
       </c>
       <c r="I20">
         <v>220</v>
@@ -1035,10 +1035,10 @@
         <v>ALL</v>
       </c>
       <c r="G21" t="str">
-        <v>Other</v>
+        <v>Trading</v>
       </c>
       <c r="H21" t="str">
-        <v>NON-Inv</v>
+        <v>Market Data</v>
       </c>
       <c r="I21">
         <v>140</v>
@@ -1064,10 +1064,10 @@
         <v>ALL</v>
       </c>
       <c r="G22" t="str">
-        <v>Other</v>
+        <v>Trading</v>
       </c>
       <c r="H22" t="str">
-        <v>NON-Inv</v>
+        <v>Market Data</v>
       </c>
       <c r="I22">
         <v>330</v>
@@ -1096,7 +1096,7 @@
         <v>PM</v>
       </c>
       <c r="H23" t="str">
-        <v>Portfolio Management</v>
+        <v>Portfolio Construction</v>
       </c>
       <c r="I23">
         <v>410</v>
@@ -1122,10 +1122,10 @@
         <v>Inv</v>
       </c>
       <c r="G24" t="str">
-        <v>PM</v>
+        <v>Other</v>
       </c>
       <c r="H24" t="str">
-        <v>Portfolio Management</v>
+        <v>Reporting &amp; MI</v>
       </c>
       <c r="I24">
         <v>30</v>
@@ -1154,7 +1154,7 @@
         <v>Other</v>
       </c>
       <c r="H25" t="str">
-        <v>NON-Inv</v>
+        <v>Reporting &amp; MI</v>
       </c>
       <c r="I25">
         <v>190</v>
@@ -1183,7 +1183,7 @@
         <v>Research</v>
       </c>
       <c r="H26" t="str">
-        <v>All</v>
+        <v>Research &amp; Analytics</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -1212,7 +1212,7 @@
         <v>PM</v>
       </c>
       <c r="H27" t="str">
-        <v>Manage Portfolio</v>
+        <v>Optimisation</v>
       </c>
       <c r="I27">
         <v>75</v>
@@ -1238,10 +1238,10 @@
         <v>Inv &amp; Ops</v>
       </c>
       <c r="G28" t="str">
-        <v>PM</v>
+        <v>Risk</v>
       </c>
       <c r="H28" t="str">
-        <v>Portfolio Management</v>
+        <v>Risk Analytics</v>
       </c>
       <c r="I28">
         <v>1800</v>
@@ -1267,10 +1267,10 @@
         <v>Inv</v>
       </c>
       <c r="G29" t="str">
-        <v>Trading</v>
+        <v>PM</v>
       </c>
       <c r="H29" t="str">
-        <v>Execution</v>
+        <v>Order Management</v>
       </c>
       <c r="I29">
         <v>1100</v>
@@ -1299,7 +1299,7 @@
         <v>Research</v>
       </c>
       <c r="H30" t="str">
-        <v>All</v>
+        <v>Research &amp; Analytics</v>
       </c>
       <c r="I30">
         <v>520</v>
@@ -1325,10 +1325,10 @@
         <v>Inv</v>
       </c>
       <c r="G31" t="str">
-        <v>Research</v>
+        <v>Trading</v>
       </c>
       <c r="H31" t="str">
-        <v>All</v>
+        <v>Market Data</v>
       </c>
       <c r="I31">
         <v>340</v>
@@ -1360,7 +1360,7 @@
         <v>PM</v>
       </c>
       <c r="H32" t="str">
-        <v>Manage Portfolio</v>
+        <v>Cash Management</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -1392,7 +1392,7 @@
         <v>PM</v>
       </c>
       <c r="H33" t="str">
-        <v>Manage Portfolio</v>
+        <v>Cash Management</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -1421,7 +1421,7 @@
         <v>Research</v>
       </c>
       <c r="H34" t="str">
-        <v>All</v>
+        <v>Research &amp; Analytics</v>
       </c>
       <c r="I34">
         <v>210</v>
@@ -1450,7 +1450,7 @@
         <v>Research</v>
       </c>
       <c r="H35" t="str">
-        <v>All</v>
+        <v>ESG</v>
       </c>
       <c r="I35">
         <v>160</v>
@@ -1537,7 +1537,7 @@
         <v>Other</v>
       </c>
       <c r="H38" t="str">
-        <v>Tech</v>
+        <v>Data Platform</v>
       </c>
       <c r="I38">
         <v>950</v>
@@ -1566,7 +1566,7 @@
         <v>Other</v>
       </c>
       <c r="H39" t="str">
-        <v>Tech</v>
+        <v>Data Platform</v>
       </c>
       <c r="I39">
         <v>480</v>
@@ -1595,7 +1595,7 @@
         <v>Other</v>
       </c>
       <c r="H40" t="str">
-        <v>Tech</v>
+        <v>Integration</v>
       </c>
       <c r="I40">
         <v>260</v>
@@ -1624,7 +1624,7 @@
         <v>Other</v>
       </c>
       <c r="H41" t="str">
-        <v>Tech</v>
+        <v>Integration</v>
       </c>
       <c r="I41">
         <v>310</v>
@@ -1653,7 +1653,7 @@
         <v>Research</v>
       </c>
       <c r="H42" t="str">
-        <v>All</v>
+        <v>Research &amp; Analytics</v>
       </c>
       <c r="I42">
         <v>400</v>
@@ -1679,10 +1679,10 @@
         <v>Inv</v>
       </c>
       <c r="G43" t="str">
-        <v>PM</v>
+        <v>Risk</v>
       </c>
       <c r="H43" t="str">
-        <v>Manage Portfolio</v>
+        <v>Risk Analytics</v>
       </c>
       <c r="I43">
         <v>230</v>
@@ -1711,7 +1711,7 @@
         <v>Other</v>
       </c>
       <c r="H44" t="str">
-        <v>Tech</v>
+        <v>Data Platform</v>
       </c>
       <c r="I44">
         <v>120</v>
@@ -1740,7 +1740,7 @@
         <v>Other</v>
       </c>
       <c r="H45" t="str">
-        <v>Tech</v>
+        <v>Data Platform</v>
       </c>
       <c r="I45">
         <v>560</v>
@@ -1769,7 +1769,7 @@
         <v>Other</v>
       </c>
       <c r="H46" t="str">
-        <v>NON-Inv</v>
+        <v>Reporting &amp; MI</v>
       </c>
       <c r="I46">
         <v>180</v>
@@ -1807,16 +1807,84 @@
         <v>Foundation</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Trade Surveillance Portal</v>
+      </c>
+      <c r="B48" t="str">
+        <v>?</v>
+      </c>
+      <c r="C48" t="str">
+        <v>In-house</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Inv &amp; Ops</v>
+      </c>
+      <c r="I48">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Collateral Manager</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Y</v>
+      </c>
+      <c r="C49" t="str">
+        <v>In-house</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Ops</v>
+      </c>
+      <c r="I49">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Index Data Loader</v>
+      </c>
+      <c r="B50" t="str">
+        <v>N</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Group Technology</v>
+      </c>
+      <c r="E50" t="str">
+        <v>ALL</v>
+      </c>
+      <c r="I50">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Client Reporting Studio</v>
+      </c>
+      <c r="B51" t="str">
+        <v>?</v>
+      </c>
+      <c r="C51" t="str">
+        <v>In-house</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Distn</v>
+      </c>
+      <c r="I51">
+        <v>95</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J51"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C46"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1902,15 +1970,15 @@
         <v>Cap L2</v>
       </c>
       <c r="B9" t="str">
-        <v>Other</v>
+        <v>Risk</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Cap L3</v>
+        <v>Cap L2</v>
       </c>
       <c r="B10" t="str">
-        <v>Portfolio Management</v>
+        <v>Other</v>
       </c>
     </row>
     <row r="11">
@@ -1918,7 +1986,10 @@
         <v>Cap L3</v>
       </c>
       <c r="B11" t="str">
-        <v>Manage Portfolio</v>
+        <v>Order Management</v>
+      </c>
+      <c r="C11" t="str">
+        <v>PM</v>
       </c>
     </row>
     <row r="12">
@@ -1926,7 +1997,10 @@
         <v>Cap L3</v>
       </c>
       <c r="B12" t="str">
-        <v>Execution</v>
+        <v>Portfolio Construction</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PM</v>
       </c>
     </row>
     <row r="13">
@@ -1934,7 +2008,10 @@
         <v>Cap L3</v>
       </c>
       <c r="B13" t="str">
-        <v>All</v>
+        <v>Optimisation</v>
+      </c>
+      <c r="C13" t="str">
+        <v>PM</v>
       </c>
     </row>
     <row r="14">
@@ -1942,7 +2019,10 @@
         <v>Cap L3</v>
       </c>
       <c r="B14" t="str">
-        <v>NON-Inv</v>
+        <v>Cash Management</v>
+      </c>
+      <c r="C14" t="str">
+        <v>PM</v>
       </c>
     </row>
     <row r="15">
@@ -1950,175 +2030,178 @@
         <v>Cap L3</v>
       </c>
       <c r="B15" t="str">
-        <v>Tech</v>
+        <v>Execution</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Trading</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Users</v>
+        <v>Cap L3</v>
       </c>
       <c r="B16" t="str">
-        <v>Inv</v>
+        <v>Market Data</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Trading</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Users</v>
+        <v>Cap L3</v>
       </c>
       <c r="B17" t="str">
-        <v>Ops</v>
+        <v>Research &amp; Analytics</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Research</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Users</v>
+        <v>Cap L3</v>
       </c>
       <c r="B18" t="str">
-        <v>Distn</v>
+        <v>ESG</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Research</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Users</v>
+        <v>Cap L3</v>
       </c>
       <c r="B19" t="str">
-        <v>ALL</v>
+        <v>Risk Analytics</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Risk</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Desk</v>
+        <v>Cap L3</v>
       </c>
       <c r="B20" t="str">
-        <v>Active Fixed Income</v>
+        <v>Data Platform</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Other</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Desk</v>
+        <v>Cap L3</v>
       </c>
       <c r="B21" t="str">
-        <v>Index Equity</v>
+        <v>Integration</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Other</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Desk</v>
+        <v>Cap L3</v>
       </c>
       <c r="B22" t="str">
-        <v>LDI &amp; Solutions</v>
+        <v>Reporting &amp; MI</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Other</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Desk</v>
+        <v>Cap L3</v>
       </c>
       <c r="B23" t="str">
-        <v>Multi-Asset</v>
+        <v>NON-Inv</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Other</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Desk</v>
+        <v>Users</v>
       </c>
       <c r="B24" t="str">
-        <v>Cash &amp; Liquidity</v>
+        <v>Inv</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Desk</v>
+        <v>Users</v>
       </c>
       <c r="B25" t="str">
-        <v>Real Assets</v>
+        <v>Ops</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Strategy</v>
+        <v>Users</v>
       </c>
       <c r="B26" t="str">
-        <v>Global Credit</v>
-      </c>
-      <c r="C26" t="str">
-        <v>Active Fixed Income</v>
+        <v>Distn</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Strategy</v>
+        <v>Users</v>
       </c>
       <c r="B27" t="str">
-        <v>Emerging Market Debt</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Active Fixed Income</v>
+        <v>ALL</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Strategy</v>
+        <v>Desk</v>
       </c>
       <c r="B28" t="str">
-        <v>Sovereign Rates</v>
-      </c>
-      <c r="C28" t="str">
         <v>Active Fixed Income</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Strategy</v>
+        <v>Desk</v>
       </c>
       <c r="B29" t="str">
-        <v>Developed Index</v>
-      </c>
-      <c r="C29" t="str">
         <v>Index Equity</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Strategy</v>
+        <v>Desk</v>
       </c>
       <c r="B30" t="str">
-        <v>Factor Index</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Index Equity</v>
+        <v>LDI &amp; Solutions</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Strategy</v>
+        <v>Desk</v>
       </c>
       <c r="B31" t="str">
-        <v>Pension Hedging</v>
-      </c>
-      <c r="C31" t="str">
-        <v>LDI &amp; Solutions</v>
+        <v>Multi-Asset</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Strategy</v>
+        <v>Desk</v>
       </c>
       <c r="B32" t="str">
-        <v>Buy &amp; Maintain</v>
-      </c>
-      <c r="C32" t="str">
-        <v>LDI &amp; Solutions</v>
+        <v>Cash &amp; Liquidity</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Strategy</v>
+        <v>Desk</v>
       </c>
       <c r="B33" t="str">
-        <v>Diversified Growth</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Multi-Asset</v>
+        <v>Real Assets</v>
       </c>
     </row>
     <row r="34">
@@ -2126,10 +2209,10 @@
         <v>Strategy</v>
       </c>
       <c r="B34" t="str">
-        <v>Retirement Income</v>
+        <v>Global Credit</v>
       </c>
       <c r="C34" t="str">
-        <v>Multi-Asset</v>
+        <v>Active Fixed Income</v>
       </c>
     </row>
     <row r="35">
@@ -2137,10 +2220,10 @@
         <v>Strategy</v>
       </c>
       <c r="B35" t="str">
-        <v>Sterling Liquidity</v>
+        <v>Emerging Market Debt</v>
       </c>
       <c r="C35" t="str">
-        <v>Cash &amp; Liquidity</v>
+        <v>Active Fixed Income</v>
       </c>
     </row>
     <row r="36">
@@ -2148,10 +2231,10 @@
         <v>Strategy</v>
       </c>
       <c r="B36" t="str">
-        <v>Short-Term Credit</v>
+        <v>Sovereign Rates</v>
       </c>
       <c r="C36" t="str">
-        <v>Cash &amp; Liquidity</v>
+        <v>Active Fixed Income</v>
       </c>
     </row>
     <row r="37">
@@ -2159,10 +2242,10 @@
         <v>Strategy</v>
       </c>
       <c r="B37" t="str">
-        <v>Private Credit</v>
+        <v>Developed Index</v>
       </c>
       <c r="C37" t="str">
-        <v>Real Assets</v>
+        <v>Index Equity</v>
       </c>
     </row>
     <row r="38">
@@ -2170,15 +2253,103 @@
         <v>Strategy</v>
       </c>
       <c r="B38" t="str">
+        <v>Factor Index</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Index Equity</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Pension Hedging</v>
+      </c>
+      <c r="C39" t="str">
+        <v>LDI &amp; Solutions</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Buy &amp; Maintain</v>
+      </c>
+      <c r="C40" t="str">
+        <v>LDI &amp; Solutions</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Diversified Growth</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Multi-Asset</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Retirement Income</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Multi-Asset</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Sterling Liquidity</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Cash &amp; Liquidity</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Short-Term Credit</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Cash &amp; Liquidity</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Private Credit</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Real Assets</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="B46" t="str">
         <v>Property Debt</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C46" t="str">
         <v>Real Assets</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C46"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5163,7 +5334,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6177,9 +6348,101 @@
         <v>Tier 2</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>APP-6120</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Trade Surveillance Portal</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Application</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Investments</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Tier 2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>APP-6184</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Collateral Manager</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Application</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Investments</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Investment Management</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Tier 2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>APP-6233</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Index Data Loader</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Interface</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Active</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Group Technology</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Data Services</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Tier 3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>APP-6297</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Client Reporting Studio</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Application</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Plan</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Investments</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Data Services</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Tier 3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>